<commit_message>
kyste hydatique du foie 1
</commit_message>
<xml_diff>
--- a/public/instruments_inventory.xlsx
+++ b/public/instruments_inventory.xlsx
@@ -24,6 +24,7 @@
     <sheet name="GOITRE 2" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="GOITRE 1" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="DCN 1" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="KYSTE HYDATIQUE DU FOIE 1" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5763,6 +5764,922 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KYSTE HYDATIQUE DU FOIE 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Réf</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Libellé</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>47506</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>VALVE LERICHE BUGATTI            45 X 260 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>02004</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>BISTOURI MANCHE N 4 LONG POUR LAMES FIG 18-19-20-21-22-23-24-25-36</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>02002</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>BISTOURI MANCHE N 3 LONG POUR LAMES FIG 10-11-12-12d-13-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>52929</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>ECARTEUR MALLEABLE HABERER 37/45 X 300 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>30914</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>PINCE DISS.  STAND. DELIC. 250 MM SS GR</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>30935</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>PINCE DISS.  STAND. NORMA. 200 MM SS GR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>30007</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>PINCE DISS.  DEBAKEY 3.5   240 MM DRT ATRAUMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>30909</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>PINCE DISS.  STAND. DELIC. 180 MM A  GR</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>17810</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>ECARTEUR DBL US ARMY 15 X 33 ET 16 X 46 210 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>02728</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>CANULE ASPIR. YANKAUER          260 MM D. 9 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>N867</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>ECARTEUR ABDOM. BALFOUR OUV.200 LT.100 M.100X70</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>47213</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>VALVE DOYEN VAGINALE             60 X 120 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>47210</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>VALVE DOYEN VAGINALE             45 X 120 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>17809</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>58011</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>TROCART OSCHNER VESICULE CH 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>N867</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>ECARTEUR ABDOM. BALFOUR OUV.200 LT.100 M.100X70</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>35405</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>PINCE HEM. KOCHER          180 MM D.AG</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>35405</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>PINCE HEM. KOCHER          180 MM D.AG</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>34203</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>PINCE HEM. BENGOLEA        210 MM C.SG</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>35101</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>PINCE HEM. KELLY           140 MM C.SG</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>35103</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>PINCE HEM. KELLY           160 MM C.SG</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>35513</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>PINCE HEM. LERICHE         150 MM C.SG</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>2032</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>37705</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>PINCE PANSEM. GROSS MAIER    250 MM DRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>35513</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>PINCE HEM. LERICHE         150 MM C.SG</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>26712</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>PASSE FILS OSHAUGN.FIN  240 MM CDE 90°</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>2032</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>26710</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>PASSE FILS OSHAUGN.FIN  220 MM CDE 90°</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>35513</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>PINCE HEM. LERICHE         150 MM C.SG</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>34203</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>PINCE HEM. BENGOLEA        210 MM C.SG</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>38902</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>PINCE PREHENS. MULTIGR. ALLIS  150 MM   5 X  6</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>35103</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>PINCE HEM. KELLY           160 MM C.SG</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>34203</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>PINCE HEM. BENGOLEA        210 MM C.SG</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>38903</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>PINCE PREHENS. MULTIGR. ALLIS  190 MM    5 X 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>38903</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>PINCE PREHENS. MULTIGR. ALLIS  190 MM    5 X 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>34202</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>PINCE HEM. BENGOLEA        210 MM D.AG</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>38903</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>PINCE PREHENS. MULTIGR. ALLIS  190 MM    5 X 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>37607</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>PINCE PANSEM. FOERSTER STRIE 250 MM DTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>37607</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>PINCE PANSEM. FOERSTER STRIE 250 MM DTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>37609</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>PINCE PANSEM. FOERSTER STRIEE 200 MM DRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>37609</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>PINCE PANSEM. FOERSTER STRIEE 200 MM DRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>UC4308</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>CISEAUX UP-CUT METZENBAUM 230 MM CBE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>UC4308</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>CISEAUX UP-CUT METZENBAUM 230 MM CBE</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>UC4304</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>CISEAUX UP-CUT METZENBAUM 180 MM CBE</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>UC4306</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>CISEAUX UP-CUT METZENBAUM 200 MM CBE</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>UN140</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>UP-NEEDLE MAYO HEGAR            200 MM       1/0 A 4/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>UN145</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>UP-NEEDLE MAYO HEGAR            240 MM       1/0 A 4/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>UN130</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>UP-NEEDLE MAYO HEGAR            180 MM       1/0 A 4/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>28402</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>PINCE CHAMPS BACKAUS 120 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>28402</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>PINCE CHAMPS BACKAUS 120 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>28402</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>PINCE CHAMPS BACKAUS 120 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>28402</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>PINCE CHAMPS BACKAUS 120 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>28402</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>PINCE CHAMPS BACKAUS 120 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>28402</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>PINCE CHAMPS BACKAUS 120 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>52206</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>HARICOT INOX 200 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>K1008</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>CUPULE INOX  D. 100 MM CAPACITE 325CC</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>K1301</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>CUPULE INOX D. 150 MM CAPACITE 900CC</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>02602</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>CADRE EPINGLE PORTE PINCES  150 MM A BOULE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
curetage 3 and 4
</commit_message>
<xml_diff>
--- a/public/instruments_inventory.xlsx
+++ b/public/instruments_inventory.xlsx
@@ -26,6 +26,8 @@
     <sheet name="DCN 1" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="KYSTE HYDATIQUE DU FOIE 1" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="MINI FRAG 2" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="CURETAGE 3" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="CURETAGE 4" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8074,6 +8076,623 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CURETAGE 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Réf</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Libellé</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>K1008</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>CUPULE INOX  D. 100 MM CAPACITE 325CC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>45505</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>SPECULUM GYNECO COLLIN            35 X 105 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>K1230</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>VALVE AUVARD            83 X 38 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>14817</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>CURETTE GYNECO GOURDET MOUSSE      260 X 10 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>14815</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>CURETTE GYNECO GOURDET MOUSSE      260 X   6 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>37607</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>PINCE PANSEM. FOERSTER STRIE 250 MM DTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>37705</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>PINCE PANSEM. GROSS MAIER    250 MM DRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>14816</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>CURETTE GYNECO GOURDET MOUSSE      260 X   8 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>14814</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>CURETTE GYNECO GOURDET MOUSSE      260 X   4 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>27503</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>PINCE BIOPSIE GYNECO DOUAY                                250 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>25514</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>HYSTEROMETRE SIMS   RIGIDE                330 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>02149</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>BOUGIE HEGAR DOUBLE SERIE EN BOITE N° 3-4 A 17-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>02149</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>BOUGIE HEGAR DOUBLE SERIE EN BOITE N° 3-4 A 17-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>02149</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>BOUGIE HEGAR DOUBLE SERIE EN BOITE N° 3-4 A 17-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>02149</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>BOUGIE HEGAR DOUBLE SERIE EN BOITE N° 3-4 A 17-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>02149</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>BOUGIE HEGAR DOUBLE SERIE EN BOITE N° 3-4 A 17-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>02149</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>BOUGIE HEGAR DOUBLE SERIE EN BOITE N° 3-4 A 17-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>02149</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>BOUGIE HEGAR DOUBLE SERIE EN BOITE N° 3-4 A 17-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>02149</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>BOUGIE HEGAR DOUBLE SERIE EN BOITE N° 3-4 A 17-18</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CURETAGE 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Réf</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Libellé</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>K1008</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>CUPULE INOX  D. 100 MM CAPACITE 325CC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>02149</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>BOUGIE HEGAR DOUBLE SERIE EN BOITE N° 3-4 A 17-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>02149</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>BOUGIE HEGAR DOUBLE SERIE EN BOITE N° 3-4 A 17-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>02149</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>BOUGIE HEGAR DOUBLE SERIE EN BOITE N° 3-4 A 17-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>02149</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>BOUGIE HEGAR DOUBLE SERIE EN BOITE N° 3-4 A 17-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>02149</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>BOUGIE HEGAR DOUBLE SERIE EN BOITE N° 3-4 A 17-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>02149</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>BOUGIE HEGAR DOUBLE SERIE EN BOITE N° 3-4 A 17-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>K1230</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>VALVE AUVARD            83 X 38 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>45506</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>SPECULUM GYNECO COLLIN            38 X 105 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>37607</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>PINCE PANSEM. FOERSTER STRIE 250 MM DTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>37804</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>PINCE PANSEM. LONGUETTE   240 MM CDE CHERON</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>33801</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>PINCE GYNECO POZZI            240 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>14815</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>CURETTE GYNECO GOURDET MOUSSE      260 X   6 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>14816</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>CURETTE GYNECO GOURDET MOUSSE      260 X   8 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>14816</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>CURETTE GYNECO GOURDET MOUSSE      260 X   8 MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>25501</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>HYSTEROMETRE SIMS    MALLEABLE                  330 MM</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
artro 1 and 2
</commit_message>
<xml_diff>
--- a/public/instruments_inventory.xlsx
+++ b/public/instruments_inventory.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3" showHorizontalScroll="1" showVerticalScroll="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="32"/>
   </bookViews>
   <sheets>
     <sheet name="CESARIENNE 2" sheetId="1" state="visible" r:id="rId1"/>
@@ -38,16 +38,15 @@
     <sheet name="ABDOMEN ENFANT 1" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="PROCTO 1" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="PROCTO 2" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="ARTRO 1" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="ARTRO 2" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="647">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="658">
   <si>
     <t xml:space="preserve">CESARIENNE 2</t>
   </si>
@@ -1988,6 +1987,39 @@
   </si>
   <si>
     <t xml:space="preserve">SONDE CANNELEE MODELE COURBE 140 MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTRO 1</t>
+  </si>
+  <si>
+    <t>31175RE.2RE</t>
+  </si>
+  <si>
+    <t>36124</t>
+  </si>
+  <si>
+    <t>39712</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PORTE AIG. DEBAKEY                 230 MM TUNGST</t>
+  </si>
+  <si>
+    <t>S3431XA.SL</t>
+  </si>
+  <si>
+    <t>S3431XB.UL</t>
+  </si>
+  <si>
+    <t>S3431XC.UM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTRO 2</t>
+  </si>
+  <si>
+    <t>S3431XB</t>
+  </si>
+  <si>
+    <t>S3431XB.UR</t>
   </si>
 </sst>
 </file>
@@ -2570,14 +2602,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2940,14 +2972,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>226</v>
       </c>
@@ -3321,14 +3353,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>252</v>
       </c>
@@ -3757,14 +3789,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>270</v>
       </c>
@@ -4248,14 +4280,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>290</v>
       </c>
@@ -4761,14 +4793,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>297</v>
       </c>
@@ -5175,14 +5207,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>300</v>
       </c>
@@ -5655,14 +5687,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>305</v>
       </c>
@@ -6223,14 +6255,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>349</v>
       </c>
@@ -6747,14 +6779,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>359</v>
       </c>
@@ -7095,14 +7127,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>403</v>
       </c>
@@ -7773,14 +7805,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>48</v>
       </c>
@@ -8154,14 +8186,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>421</v>
       </c>
@@ -8808,14 +8840,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>478</v>
       </c>
@@ -9057,14 +9089,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>493</v>
       </c>
@@ -9273,14 +9305,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>496</v>
       </c>
@@ -9522,14 +9554,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>517</v>
       </c>
@@ -9782,14 +9814,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>520</v>
       </c>
@@ -9932,14 +9964,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>521</v>
       </c>
@@ -10434,14 +10466,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>563</v>
       </c>
@@ -10595,14 +10627,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>566</v>
       </c>
@@ -11988,7 +12020,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
-    <col customWidth="1" min="3" max="3" width="66.421875"/>
+    <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
     <row r="1" ht="21">
@@ -12369,7 +12401,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
-    <col customWidth="1" min="3" max="3" width="65.28125"/>
+    <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
     <row r="1" ht="21">
@@ -12706,7 +12738,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
-    <col customWidth="1" min="3" max="3" width="65.57421875"/>
+    <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
     <row r="1" ht="21">
@@ -13040,6 +13072,460 @@
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="8"/>
+    <col customWidth="1" min="2" max="2" width="15"/>
+    <col customWidth="1" min="3" max="3" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="21">
+      <c r="A1" s="1" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>8</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3">
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>648</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>649</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>650</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>652</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3">
+        <v>14</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>653</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3">
+        <v>15</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>653</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3">
+        <v>16</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="8"/>
+    <col customWidth="1" min="2" max="2" width="15"/>
+    <col customWidth="1" min="3" max="3" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="21">
+      <c r="A1" s="1" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>8</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>648</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3">
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>649</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>649</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>652</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3">
+        <v>14</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>656</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3">
+        <v>15</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>657</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3">
+        <v>16</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>
@@ -13054,7 +13540,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
-    <col customWidth="1" min="3" max="3" width="65.28125"/>
+    <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
     <row r="1" ht="21">
@@ -13442,14 +13928,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>73</v>
       </c>
@@ -14175,14 +14661,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>130</v>
       </c>
@@ -14930,14 +15416,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>171</v>
       </c>
@@ -15652,14 +16138,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>178</v>
       </c>
@@ -16330,14 +16816,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>215</v>
       </c>

</xml_diff>

<commit_message>
orthopedie rachis lambaire 1
</commit_message>
<xml_diff>
--- a/public/instruments_inventory.xlsx
+++ b/public/instruments_inventory.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="33"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="28"/>
   </bookViews>
   <sheets>
     <sheet name="CESARIENNE 2" sheetId="1" state="visible" r:id="rId1"/>
@@ -35,19 +35,20 @@
     <sheet name="RHINOPLASTIE 1" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="CERCLAGE 4" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="ORTHOPEDIE MS 1" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="ABDOMEN ENFANT 1" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="PROCTO 1" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="PROCTO 2" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="ARTRO 1" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="ARTRO 2" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="COLPOSCOPIE CONSULTATION GYNECO" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="ORTHOPEDIE RACHIS LAMBAIRE 1" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="ABDOMEN ENFANT 1" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="PROCTO 1" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="PROCTO 2" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="ARTRO 1" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="ARTRO 2" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="COLPOSCOPIE CONSULTATION GYNECO" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="659">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="746">
   <si>
     <t xml:space="preserve">CESARIENNE 2</t>
   </si>
@@ -1918,6 +1919,279 @@
     <t xml:space="preserve">DAVIER OS VERBRUGGE REDUCT. AUTO CENTR.  240 MM</t>
   </si>
   <si>
+    <t xml:space="preserve">ORTHOPEDIE RACHIS LAMBAIRE 1</t>
+  </si>
+  <si>
+    <t>01215</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALENE REDON COURBE CH 14 DIAM 4,6 MM</t>
+  </si>
+  <si>
+    <t>02723</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CANULE ASPIR. WERTHEIMER RIG.CD 170 MM D. 3 MM</t>
+  </si>
+  <si>
+    <t>14001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CROCHET CUSHING         190 MM FIN  MSSE 4 MM</t>
+  </si>
+  <si>
+    <t>14003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CROCHET CUSHING         190 MM FORT MSSE 6 MM</t>
+  </si>
+  <si>
+    <t>14006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CROCHET DANDY            230 MM MSSE DROIT</t>
+  </si>
+  <si>
+    <t>15720</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CURETTE OSS. CLOWARD DROITE           200 X  4.8 MM FIG 3</t>
+  </si>
+  <si>
+    <t>17105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DISSECTEUR DAVIS 245 MM UN COTE TRANCHANT 6 MM UN COTE MOUSSE  6,8 MM </t>
+  </si>
+  <si>
+    <t>17201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DISSECTEUR FREER 200 MM  1 COTE MOUSSE 5MM 1 COTE TRANCHANT 4,5 MM</t>
+  </si>
+  <si>
+    <t>19002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECARTEUR /MANCHE LOVE        COUDE 45° 190 MM</t>
+  </si>
+  <si>
+    <t>19003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECARTEUR /MANCHE LOVE        COUDE 90° 190 MM</t>
+  </si>
+  <si>
+    <t>2029</t>
+  </si>
+  <si>
+    <t>21807</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECARTEUR AUT.ADSON BECKMANN 320 MM MSS 25X38</t>
+  </si>
+  <si>
+    <t>21910</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECARTEUR AUT.BECKMANN      MSS    50X 300 MM</t>
+  </si>
+  <si>
+    <t>22009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECARTEUR AUT.BECKMANN STILLE MSS     35X 330 MM</t>
+  </si>
+  <si>
+    <t>22803</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECARTEUR AUT.WEITLANER GR. MSS 3 X 4  130 MM</t>
+  </si>
+  <si>
+    <t>23606</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECARTEUR AUT.RACH. SCOV. HAVERFIELD  150 MM SEUL</t>
+  </si>
+  <si>
+    <t>29007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PINCE COUPANTE DBL ART. LISTON KEY HORSLEY 260 MM          </t>
+  </si>
+  <si>
+    <t>32603</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PINCE GOUGE DBL ART. LEKSELL    230 X  8MM</t>
+  </si>
+  <si>
+    <t>32902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PINCE GOUGE DBL ART. SMITH PETERSEN 230 MM CBE</t>
+  </si>
+  <si>
+    <t>34302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PINCE HEM. BENGOLEA        240 MM FINE     C.SG UPLINE</t>
+  </si>
+  <si>
+    <t>39712</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PORTE AIG. DEBAKEY                 230 MM TUNGST</t>
+  </si>
+  <si>
+    <t>41901</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONGEUR DISQUE FERRIS        180 CDE BAS 2X10</t>
+  </si>
+  <si>
+    <t>41902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONGEUR DISQUE FERRIS        180 CDE HT  2X10</t>
+  </si>
+  <si>
+    <t>41903</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONGEUR DISQUE FERRIS        180 DROIT   2X10</t>
+  </si>
+  <si>
+    <t>41904</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONGEUR DISQUE FERRIS        180 CDE BAS 3X10</t>
+  </si>
+  <si>
+    <t>41905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONGEUR DISQUE FERRIS        180 CDE HT  3X10</t>
+  </si>
+  <si>
+    <t>41906</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONGEUR DISQUE FERRIS        180 DROIT   3X10</t>
+  </si>
+  <si>
+    <t>41907</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONGEUR DISQUE FERRIS        180 CDE BAS 4X10</t>
+  </si>
+  <si>
+    <t>41908</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONGEUR DISQUE FERRIS        180 CDE HT  4X10</t>
+  </si>
+  <si>
+    <t>41912C</t>
+  </si>
+  <si>
+    <t>42106C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONGEUR DISQUE SPURLING CERAM.180 CDE HT  4X10</t>
+  </si>
+  <si>
+    <t>42305C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONGEUR LAMINA CERAM.PM 180 X 1 MM 40° HT  DEM.</t>
+  </si>
+  <si>
+    <t>42308C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONGEUR LAMINA CERAM.PM 180 X 2 MM 40° HT  DEM.</t>
+  </si>
+  <si>
+    <t>42313C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONGEUR LAMINA CERAM.PM 180 X 3 MM 40° HT  DEM.</t>
+  </si>
+  <si>
+    <t>42319C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONGEUR LAMINA CERAM.PM 200 X 5 MM 90° HT  DEM.</t>
+  </si>
+  <si>
+    <t>42331C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONGEUR LAMINA CERAM.PM 200 X 4 MM 40° HT  DEM.</t>
+  </si>
+  <si>
+    <t>43013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUGINE COBB RACHIS MCHE ROND   240 X 19 MM</t>
+  </si>
+  <si>
+    <t>43309</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUGINE LAMBOTTE                   25 X 210 MM</t>
+  </si>
+  <si>
+    <t>54307</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAILLET WILLIGER 26X240MM 300g REMPL PLOMB</t>
+  </si>
+  <si>
+    <t>K632</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIS. OS OSTEOT. LAMBOTTE             8 X 240 MM LAME FINE</t>
+  </si>
+  <si>
+    <t>UC4306C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CISEAUX UP-CUT METZENBAUM 200 MM CBE CERAM</t>
+  </si>
+  <si>
+    <t>UC4308C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CISEAUX UP-CUT METZENBAUM 230 MM CBE CERAM</t>
+  </si>
+  <si>
+    <t>UC4332C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CISEAUX UP-CUT MAYO STILLE 170 MM CBE CERAM</t>
+  </si>
+  <si>
+    <t>W467</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECARTEUR /MANCHE KOCHER 230 MM 60 X 25 MM</t>
+  </si>
+  <si>
+    <t>W544</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIS. OS OSTEOT. LAMBOTTE           10 X 240 MM COURBE</t>
+  </si>
+  <si>
+    <t>W811</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CURETTE OSS. COBB                  280 X   8.5 MM</t>
+  </si>
+  <si>
     <t xml:space="preserve">ABDOMEN ENFANT 1</t>
   </si>
   <si>
@@ -1939,12 +2213,6 @@
     <t xml:space="preserve">PINCE DISS.  DEBAKEY 3.5   200 MM DRT ATRAUMA</t>
   </si>
   <si>
-    <t>34302</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PINCE HEM. BENGOLEA        240 MM FINE     C.SG UPLINE</t>
-  </si>
-  <si>
     <t>34906</t>
   </si>
   <si>
@@ -1997,12 +2265,6 @@
   </si>
   <si>
     <t>36124</t>
-  </si>
-  <si>
-    <t>39712</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PORTE AIG. DEBAKEY                 230 MM TUNGST</t>
   </si>
   <si>
     <t>S3431XA.SL</t>
@@ -11428,13 +11690,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
   </sheetPr>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
-    <col customWidth="1" min="3" max="3" width="60"/>
+    <col customWidth="1" min="3" max="3" width="76.00390625"/>
   </cols>
   <sheetData>
     <row r="1" ht="21">
@@ -11458,10 +11720,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>76</v>
+        <v>624</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>77</v>
+        <v>625</v>
       </c>
     </row>
     <row r="5">
@@ -11469,10 +11731,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>78</v>
+        <v>404</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>79</v>
+        <v>405</v>
       </c>
     </row>
     <row r="6">
@@ -11480,10 +11742,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>436</v>
+        <v>4</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>437</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -11491,10 +11753,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>436</v>
+        <v>6</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>437</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -11502,10 +11764,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>10</v>
+        <v>626</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>11</v>
+        <v>627</v>
       </c>
     </row>
     <row r="9">
@@ -11513,10 +11775,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>10</v>
+        <v>628</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>11</v>
+        <v>629</v>
       </c>
     </row>
     <row r="10">
@@ -11524,10 +11786,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
     </row>
     <row r="11">
@@ -11535,10 +11797,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>624</v>
+        <v>632</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>625</v>
+        <v>633</v>
       </c>
     </row>
     <row r="12">
@@ -11546,10 +11808,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>137</v>
+        <v>634</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>138</v>
+        <v>635</v>
       </c>
     </row>
     <row r="13">
@@ -11557,10 +11819,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>137</v>
+        <v>636</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>138</v>
+        <v>637</v>
       </c>
     </row>
     <row r="14">
@@ -11568,10 +11830,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>271</v>
+        <v>638</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>232</v>
+        <v>639</v>
       </c>
     </row>
     <row r="15">
@@ -11579,10 +11841,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>272</v>
+        <v>10</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>273</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16">
@@ -11590,10 +11852,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>626</v>
+        <v>10</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>627</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17">
@@ -11601,10 +11863,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>599</v>
+        <v>640</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>600</v>
+        <v>641</v>
       </c>
     </row>
     <row r="18">
@@ -11612,10 +11874,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>298</v>
+        <v>642</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>299</v>
+        <v>643</v>
       </c>
     </row>
     <row r="19">
@@ -11623,10 +11885,10 @@
         <v>16</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>14</v>
+        <v>644</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>15</v>
+        <v>232</v>
       </c>
     </row>
     <row r="20">
@@ -11634,10 +11896,10 @@
         <v>17</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>14</v>
+        <v>406</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>15</v>
+        <v>232</v>
       </c>
     </row>
     <row r="21">
@@ -11645,10 +11907,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>14</v>
+        <v>645</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>15</v>
+        <v>646</v>
       </c>
     </row>
     <row r="22">
@@ -11656,10 +11918,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>14</v>
+        <v>647</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>15</v>
+        <v>648</v>
       </c>
     </row>
     <row r="23">
@@ -11667,10 +11929,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>14</v>
+        <v>649</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>15</v>
+        <v>650</v>
       </c>
     </row>
     <row r="24">
@@ -11678,10 +11940,10 @@
         <v>21</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>143</v>
+        <v>651</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>144</v>
+        <v>652</v>
       </c>
     </row>
     <row r="25">
@@ -11689,10 +11951,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>628</v>
+        <v>653</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>629</v>
+        <v>654</v>
       </c>
     </row>
     <row r="26">
@@ -11700,10 +11962,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>52</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27">
@@ -11711,10 +11973,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>295</v>
+        <v>14</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>296</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28">
@@ -11722,10 +11984,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>56</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29">
@@ -11733,10 +11995,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>56</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30">
@@ -11744,10 +12006,10 @@
         <v>27</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>630</v>
+        <v>14</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>631</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31">
@@ -11755,10 +12017,10 @@
         <v>28</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>632</v>
+        <v>655</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>633</v>
+        <v>656</v>
       </c>
     </row>
     <row r="32">
@@ -11766,10 +12028,10 @@
         <v>29</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>464</v>
+        <v>301</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>465</v>
+        <v>302</v>
       </c>
     </row>
     <row r="33">
@@ -11777,10 +12039,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>147</v>
+        <v>53</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>148</v>
+        <v>54</v>
       </c>
     </row>
     <row r="34">
@@ -11788,10 +12050,10 @@
         <v>31</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>147</v>
+        <v>218</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>148</v>
+        <v>219</v>
       </c>
     </row>
     <row r="35">
@@ -11799,10 +12061,10 @@
         <v>32</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>147</v>
+        <v>657</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>148</v>
+        <v>658</v>
       </c>
     </row>
     <row r="36">
@@ -11810,10 +12072,10 @@
         <v>33</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>22</v>
+        <v>659</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>23</v>
+        <v>660</v>
       </c>
     </row>
     <row r="37">
@@ -11821,10 +12083,10 @@
         <v>34</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>24</v>
+        <v>661</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>25</v>
+        <v>662</v>
       </c>
     </row>
     <row r="38">
@@ -11832,10 +12094,10 @@
         <v>35</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>150</v>
+        <v>23</v>
       </c>
     </row>
     <row r="39">
@@ -11843,10 +12105,10 @@
         <v>36</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>149</v>
+        <v>30</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
     </row>
     <row r="40">
@@ -11854,10 +12116,10 @@
         <v>37</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>26</v>
+        <v>663</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>27</v>
+        <v>664</v>
       </c>
     </row>
     <row r="41">
@@ -11865,10 +12127,10 @@
         <v>38</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>222</v>
+        <v>665</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>223</v>
+        <v>666</v>
       </c>
     </row>
     <row r="42">
@@ -11876,10 +12138,10 @@
         <v>39</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>330</v>
+        <v>667</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>331</v>
+        <v>668</v>
       </c>
     </row>
     <row r="43">
@@ -11887,10 +12149,10 @@
         <v>40</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>34</v>
+        <v>669</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>35</v>
+        <v>670</v>
       </c>
     </row>
     <row r="44">
@@ -11898,10 +12160,10 @@
         <v>41</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>634</v>
+        <v>671</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>635</v>
+        <v>672</v>
       </c>
     </row>
     <row r="45">
@@ -11909,10 +12171,10 @@
         <v>42</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>114</v>
+        <v>671</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>115</v>
+        <v>672</v>
       </c>
     </row>
     <row r="46">
@@ -11920,10 +12182,10 @@
         <v>43</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>250</v>
+        <v>673</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>251</v>
+        <v>674</v>
       </c>
     </row>
     <row r="47">
@@ -11931,10 +12193,10 @@
         <v>44</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>636</v>
+        <v>675</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>232</v>
+        <v>676</v>
       </c>
     </row>
     <row r="48">
@@ -11942,10 +12204,10 @@
         <v>45</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>336</v>
+        <v>677</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>337</v>
+        <v>678</v>
       </c>
     </row>
     <row r="49">
@@ -11953,10 +12215,10 @@
         <v>46</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>40</v>
+        <v>679</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>41</v>
+        <v>680</v>
       </c>
     </row>
     <row r="50">
@@ -11964,10 +12226,10 @@
         <v>47</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>71</v>
+        <v>681</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>72</v>
+        <v>232</v>
       </c>
     </row>
     <row r="51">
@@ -11975,10 +12237,10 @@
         <v>48</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>341</v>
+        <v>682</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>342</v>
+        <v>683</v>
       </c>
     </row>
     <row r="52">
@@ -11986,10 +12248,10 @@
         <v>49</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>44</v>
+        <v>684</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>45</v>
+        <v>685</v>
       </c>
     </row>
     <row r="53">
@@ -11997,10 +12259,252 @@
         <v>50</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>474</v>
+        <v>686</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>475</v>
+        <v>687</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3">
+        <v>51</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3">
+        <v>52</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3">
+        <v>53</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>692</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3">
+        <v>54</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>694</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3">
+        <v>55</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3">
+        <v>56</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3">
+        <v>57</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3">
+        <v>58</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>698</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3">
+        <v>59</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3">
+        <v>60</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3">
+        <v>61</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>700</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3">
+        <v>62</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>702</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3">
+        <v>63</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>704</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3">
+        <v>64</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3">
+        <v>65</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>706</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3">
+        <v>66</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>706</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3">
+        <v>67</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3">
+        <v>68</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3">
+        <v>69</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3">
+        <v>70</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>710</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3">
+        <v>71</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>712</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3">
+        <v>72</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>712</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>713</v>
       </c>
     </row>
   </sheetData>
@@ -12008,8 +12512,8 @@
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" scale="91" firstPageNumber="1" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>
@@ -12410,7 +12914,7 @@
   <sheetData>
     <row r="1" ht="21">
       <c r="A1" s="1" t="s">
-        <v>637</v>
+        <v>714</v>
       </c>
     </row>
     <row r="3">
@@ -12429,10 +12933,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5">
@@ -12440,10 +12944,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>14</v>
+        <v>78</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>15</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6">
@@ -12451,10 +12955,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>14</v>
+        <v>436</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>15</v>
+        <v>437</v>
       </c>
     </row>
     <row r="7">
@@ -12462,10 +12966,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>14</v>
+        <v>436</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>15</v>
+        <v>437</v>
       </c>
     </row>
     <row r="8">
@@ -12473,10 +12977,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -12484,10 +12988,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>242</v>
+        <v>10</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>243</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
@@ -12495,10 +12999,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>16</v>
+        <v>715</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>17</v>
+        <v>716</v>
       </c>
     </row>
     <row r="11">
@@ -12506,10 +13010,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>147</v>
+        <v>715</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>148</v>
+        <v>716</v>
       </c>
     </row>
     <row r="12">
@@ -12517,10 +13021,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>22</v>
+        <v>137</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>23</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13">
@@ -12528,10 +13032,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14">
@@ -12539,10 +13043,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>149</v>
+        <v>271</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>150</v>
+        <v>232</v>
       </c>
     </row>
     <row r="15">
@@ -12550,10 +13054,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>174</v>
+        <v>272</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>175</v>
+        <v>273</v>
       </c>
     </row>
     <row r="16">
@@ -12561,10 +13065,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>330</v>
+        <v>717</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>331</v>
+        <v>718</v>
       </c>
     </row>
     <row r="17">
@@ -12572,10 +13076,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>30</v>
+        <v>599</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>31</v>
+        <v>600</v>
       </c>
     </row>
     <row r="18">
@@ -12583,10 +13087,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>32</v>
+        <v>298</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>33</v>
+        <v>299</v>
       </c>
     </row>
     <row r="19">
@@ -12594,10 +13098,10 @@
         <v>16</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>108</v>
+        <v>14</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>109</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20">
@@ -12605,10 +13109,10 @@
         <v>17</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>108</v>
+        <v>14</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>109</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21">
@@ -12616,10 +13120,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>638</v>
+        <v>14</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>639</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22">
@@ -12627,10 +13131,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>640</v>
+        <v>14</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>641</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23">
@@ -12638,10 +13142,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>640</v>
+        <v>14</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>641</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24">
@@ -12649,10 +13153,10 @@
         <v>21</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>353</v>
+        <v>143</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>354</v>
+        <v>144</v>
       </c>
     </row>
     <row r="25">
@@ -12660,10 +13164,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>642</v>
+        <v>719</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>643</v>
+        <v>720</v>
       </c>
     </row>
     <row r="26">
@@ -12671,10 +13175,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>159</v>
+        <v>51</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>160</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27">
@@ -12682,10 +13186,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>40</v>
+        <v>295</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>41</v>
+        <v>296</v>
       </c>
     </row>
     <row r="28">
@@ -12693,10 +13197,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>163</v>
+        <v>55</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>164</v>
+        <v>56</v>
       </c>
     </row>
     <row r="29">
@@ -12704,10 +13208,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
     </row>
     <row r="30">
@@ -12715,10 +13219,263 @@
         <v>27</v>
       </c>
       <c r="B30" s="3" t="s">
+        <v>661</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3">
+        <v>28</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>721</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3">
+        <v>29</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3">
+        <v>30</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3">
+        <v>31</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3">
+        <v>32</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3">
+        <v>33</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3">
+        <v>34</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3">
+        <v>35</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3">
+        <v>36</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3">
+        <v>37</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3">
+        <v>38</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3">
+        <v>39</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3">
+        <v>40</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3">
+        <v>41</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>723</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3">
+        <v>42</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3">
+        <v>43</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3">
         <v>44</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="B47" s="3" t="s">
+        <v>725</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3">
         <v>45</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3">
+        <v>46</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3">
+        <v>47</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3">
+        <v>48</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3">
+        <v>49</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3">
+        <v>50</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>475</v>
       </c>
     </row>
   </sheetData>
@@ -12747,7 +13504,7 @@
   <sheetData>
     <row r="1" ht="21">
       <c r="A1" s="1" t="s">
-        <v>644</v>
+        <v>726</v>
       </c>
     </row>
     <row r="3">
@@ -12843,10 +13600,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>22</v>
+        <v>147</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>23</v>
+        <v>148</v>
       </c>
     </row>
     <row r="12">
@@ -12953,10 +13710,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>638</v>
+        <v>727</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>639</v>
+        <v>728</v>
       </c>
     </row>
     <row r="22">
@@ -12964,10 +13721,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>640</v>
+        <v>729</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>641</v>
+        <v>730</v>
       </c>
     </row>
     <row r="23">
@@ -12975,10 +13732,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>640</v>
+        <v>729</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>641</v>
+        <v>730</v>
       </c>
     </row>
     <row r="24">
@@ -12997,10 +13754,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>642</v>
+        <v>731</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>643</v>
+        <v>732</v>
       </c>
     </row>
     <row r="26">
@@ -13030,10 +13787,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>645</v>
+        <v>163</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>646</v>
+        <v>164</v>
       </c>
     </row>
     <row r="29">
@@ -13041,10 +13798,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>163</v>
+        <v>42</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>164</v>
+        <v>43</v>
       </c>
     </row>
     <row r="30">
@@ -13052,20 +13809,9 @@
         <v>27</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3">
-        <v>28</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C31" s="4" t="s">
         <v>45</v>
       </c>
     </row>
@@ -13095,7 +13841,7 @@
   <sheetData>
     <row r="1" ht="21">
       <c r="A1" s="1" t="s">
-        <v>647</v>
+        <v>733</v>
       </c>
     </row>
     <row r="3">
@@ -13114,10 +13860,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -13125,10 +13871,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>229</v>
+        <v>14</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>230</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -13169,10 +13915,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>14</v>
+        <v>242</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>15</v>
+        <v>243</v>
       </c>
     </row>
     <row r="10">
@@ -13180,10 +13926,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11">
@@ -13191,10 +13937,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12">
@@ -13202,10 +13948,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13">
@@ -13213,10 +13959,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>648</v>
+        <v>149</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>232</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14">
@@ -13224,10 +13970,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>649</v>
+        <v>149</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>232</v>
+        <v>150</v>
       </c>
     </row>
     <row r="15">
@@ -13235,10 +13981,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>650</v>
+        <v>174</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>651</v>
+        <v>175</v>
       </c>
     </row>
     <row r="16">
@@ -13246,10 +13992,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>652</v>
+        <v>330</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>232</v>
+        <v>331</v>
       </c>
     </row>
     <row r="17">
@@ -13257,10 +14003,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>653</v>
+        <v>30</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>232</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18">
@@ -13268,10 +14014,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>653</v>
+        <v>32</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>232</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19">
@@ -13279,10 +14025,142 @@
         <v>16</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>654</v>
+        <v>108</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>232</v>
+        <v>109</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>727</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3">
+        <v>19</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>729</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3">
+        <v>20</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>729</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3">
+        <v>22</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>731</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3">
+        <v>23</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3">
+        <v>24</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3">
+        <v>25</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>734</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3">
+        <v>26</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3">
+        <v>27</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3">
+        <v>28</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -13311,7 +14189,7 @@
   <sheetData>
     <row r="1" ht="21">
       <c r="A1" s="1" t="s">
-        <v>655</v>
+        <v>736</v>
       </c>
     </row>
     <row r="3">
@@ -13341,10 +14219,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>14</v>
+        <v>229</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>15</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6">
@@ -13396,10 +14274,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>143</v>
+        <v>14</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>144</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
@@ -13418,10 +14296,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>648</v>
+        <v>18</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>232</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13">
@@ -13429,7 +14307,7 @@
         <v>10</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>649</v>
+        <v>737</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>232</v>
@@ -13440,7 +14318,7 @@
         <v>11</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>649</v>
+        <v>738</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>232</v>
@@ -13451,10 +14329,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>30</v>
+        <v>663</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>31</v>
+        <v>664</v>
       </c>
     </row>
     <row r="16">
@@ -13462,7 +14340,7 @@
         <v>13</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>652</v>
+        <v>739</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>232</v>
@@ -13473,7 +14351,7 @@
         <v>14</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>656</v>
+        <v>740</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>232</v>
@@ -13484,7 +14362,7 @@
         <v>15</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>657</v>
+        <v>740</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>232</v>
@@ -13495,32 +14373,10 @@
         <v>16</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>654</v>
+        <v>741</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>232</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3">
-        <v>17</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3">
-        <v>18</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -13538,7 +14394,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
@@ -13549,7 +14405,7 @@
   <sheetData>
     <row r="1" ht="21">
       <c r="A1" s="1" t="s">
-        <v>658</v>
+        <v>742</v>
       </c>
     </row>
     <row r="3">
@@ -13568,10 +14424,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>240</v>
+        <v>8</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>241</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -13579,10 +14435,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>98</v>
+        <v>14</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>99</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -13590,10 +14446,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>98</v>
+        <v>14</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>99</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -13601,10 +14457,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>100</v>
+        <v>14</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>101</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -13612,10 +14468,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>509</v>
+        <v>14</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>510</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -13623,10 +14479,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>67</v>
+        <v>14</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>68</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -13634,10 +14490,131 @@
         <v>7</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>34</v>
+        <v>143</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>35</v>
+        <v>144</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>8</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>737</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3">
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>738</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>738</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>739</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3">
+        <v>14</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>743</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3">
+        <v>15</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>744</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3">
+        <v>16</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>741</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -13646,7 +14623,124 @@
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="8"/>
+    <col customWidth="1" min="2" max="2" width="15"/>
+    <col customWidth="1" min="3" max="3" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="21">
+      <c r="A1" s="1" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
ortho hanche 1 + 2
</commit_message>
<xml_diff>
--- a/public/instruments_inventory.xlsx
+++ b/public/instruments_inventory.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="45" showHorizontalScroll="1" showVerticalScroll="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="43" showHorizontalScroll="1" showVerticalScroll="1"/>
   </bookViews>
   <sheets>
     <sheet name="CESARIENNE 2" sheetId="1" state="visible" r:id="rId1"/>
@@ -50,9 +50,14 @@
     <sheet name="ORTHOPEDIE RACHIS LOMBAIRE 2 (TEST)" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="ORTHOPEDIE RACHIS CERBICAL 1" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="ORTHOPEDIE RACHIS CERBICAL 2" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="VASCULAIRE 1" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="HEPATOBILIAIRE 1" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="GOITRE 3" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="ORTHOPEDIE HANCHE 1" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="ORTHOPEDIE HANCHE 2" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="VASCULAIRE 1" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="HEPATOBILIAIRE 1" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="GOITRE 3" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="CURETTAGE 2" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="CURETTAGE 3" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="CURETTAGE 4" sheetId="51" state="visible" r:id="rId51"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
   <extLst>
@@ -62,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="1006">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="1068">
   <si>
     <t xml:space="preserve">CESARIENNE 2</t>
   </si>
@@ -2761,6 +2766,195 @@
     <t xml:space="preserve">PINCE GOUGE SIMPLE STELLBRINK 170X 2 MM CBE</t>
   </si>
   <si>
+    <t xml:space="preserve">ORTHOPEDIE HANCHE 1</t>
+  </si>
+  <si>
+    <t>08209</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIS. OS OSTEOT. STILLE DROIT       15 X 210 MM</t>
+  </si>
+  <si>
+    <t>08216</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIS. OS OSTEOT. STILLE COURBE   20 X 210 MM</t>
+  </si>
+  <si>
+    <t>11208</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PINCE A DISS. LIGATURE  ZENKER COURBE 290MM</t>
+  </si>
+  <si>
+    <t>14303</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CROCHET LAMBOTTE         280 MM GRAND MODELE</t>
+  </si>
+  <si>
+    <t>15618</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CURETTE OSS. BRUNS ANGULEE   230 X  6.1 MM FIG 4</t>
+  </si>
+  <si>
+    <t>15856</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CURETTE OSS. VOLKMANN              280 X 10 MM</t>
+  </si>
+  <si>
+    <t>18004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECARTEUR /MANCHE BENNET        65 MM    260 MM</t>
+  </si>
+  <si>
+    <t>18703</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECARTEUR /MANCHE HOHMANN 265 MM  24.0 MM</t>
+  </si>
+  <si>
+    <t>19605</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECARTEUR /MANCHE SIMON 27 X 115 MM</t>
+  </si>
+  <si>
+    <t>22004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECARTEUR AUT.BECKMANN CONE MSS     20X 330 MM</t>
+  </si>
+  <si>
+    <t>24602</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ELEVATEUR LAMBOTTE CUILLER DOUBLE  290 MM LARGEUR 15 ET 30MM</t>
+  </si>
+  <si>
+    <t>25812</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MASSE OMBREDANNE 230MM DIAM 40 MM 900 GR</t>
+  </si>
+  <si>
+    <t>26709</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASSE FILS OSHAUGN.FIN  220 MM CDE 45°</t>
+  </si>
+  <si>
+    <t>29004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PINCE COUPANTE DBL ART. LISTON 270 MM DROITE</t>
+  </si>
+  <si>
+    <t>30936</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PINCE DISS.  STAND. NORMA. 250 MM 1 X 2 GR</t>
+  </si>
+  <si>
+    <t>32803</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PINCE GOUGE DBL ART. RUSKIN     240 X  5MM CBE</t>
+  </si>
+  <si>
+    <t>34003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PINCE GYNECO WERTHEIM CBE A  GR            230 MM</t>
+  </si>
+  <si>
+    <t>43308</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUGINE LAMBOTTE                   20 X 210 MM</t>
+  </si>
+  <si>
+    <t>56614</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PINCE HEM. ROBERTS       220 MM C.SG</t>
+  </si>
+  <si>
+    <t>A6QK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POINTE CARREE PERTHES                  210 MM (alene)</t>
+  </si>
+  <si>
+    <t>CAXC</t>
+  </si>
+  <si>
+    <t>K536</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIS. OS GOUGE  MANCHE SYNTH.   5 X 250 MM</t>
+  </si>
+  <si>
+    <t>Z593</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DAVIER OS VERBRUGGE REDUCT. AUTO CENTR.  260 MM</t>
+  </si>
+  <si>
+    <t>Z594</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DAVIER OS VERBRUGGE REDUCT. AUTO CENTR.  280 MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORTHOPEDIE HANCHE 2</t>
+  </si>
+  <si>
+    <t>04121</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CISEAUX DISS. METZ.NELSON 250 MM CBE  TUNGST</t>
+  </si>
+  <si>
+    <t>08114</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIS. OS OSTEOT. LAMBOTTE           14 X 240 MM</t>
+  </si>
+  <si>
+    <t>08210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIS. OS OSTEOT. STILLE DROIT       20 X 210 MM</t>
+  </si>
+  <si>
+    <t>08213</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIS. OS OSTEOT. STILLE COURBE   10 X 210 MM</t>
+  </si>
+  <si>
+    <t>15855</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CURETTE OSS. VOLKMANN              280 X   8 MM</t>
+  </si>
+  <si>
+    <t>30913</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PINCE DISS.  STAND. DELIC. 250 MM A  GR</t>
+  </si>
+  <si>
+    <t>32602</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PINCE GOUGE DBL ART. LEKSELL    230 X  5MM</t>
+  </si>
+  <si>
     <t xml:space="preserve">VASCULAIRE 1</t>
   </si>
   <si>
@@ -2866,12 +3060,6 @@
     <t xml:space="preserve">ECARTEUR AUT.BECKMANN      MSS    20X 300 MM</t>
   </si>
   <si>
-    <t>22004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ECARTEUR AUT.BECKMANN CONE MSS     20X 330 MM</t>
-  </si>
-  <si>
     <t>22807</t>
   </si>
   <si>
@@ -3028,12 +3216,6 @@
     <t xml:space="preserve">PASSE FILS GEMINI 230MM</t>
   </si>
   <si>
-    <t>56614</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PINCE HEM. ROBERTS       220 MM C.SG</t>
-  </si>
-  <si>
     <t>UL130</t>
   </si>
   <si>
@@ -3080,6 +3262,15 @@
   </si>
   <si>
     <t xml:space="preserve">PINCE HEM. LERICHE         150 MM D.AG UPLINE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CURETTAGE 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CURETTAGE 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CURETTAGE 4</t>
   </si>
 </sst>
 </file>
@@ -19909,14 +20100,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
-    <col customWidth="1" min="3" max="3" width="60"/>
+    <col customWidth="1" min="3" max="3" width="68.8515625"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>899</v>
       </c>
@@ -19948,10 +20139,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>4</v>
+        <v>77</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>5</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6">
@@ -19970,10 +20161,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>7</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">
@@ -19981,10 +20172,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>900</v>
+        <v>81</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>901</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9">
@@ -19992,10 +20183,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>365</v>
+        <v>900</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>366</v>
+        <v>901</v>
       </c>
     </row>
     <row r="10">
@@ -20058,10 +20249,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>912</v>
+        <v>273</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>913</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16">
@@ -20069,10 +20260,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>914</v>
+        <v>273</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>915</v>
+        <v>274</v>
       </c>
     </row>
     <row r="17">
@@ -20080,10 +20271,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>916</v>
+        <v>912</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>917</v>
+        <v>913</v>
       </c>
     </row>
     <row r="18">
@@ -20091,10 +20282,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>918</v>
+        <v>585</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>919</v>
+        <v>586</v>
       </c>
     </row>
     <row r="19">
@@ -20102,10 +20293,10 @@
         <v>16</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>920</v>
+        <v>585</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>921</v>
+        <v>586</v>
       </c>
     </row>
     <row r="20">
@@ -20113,10 +20304,10 @@
         <v>17</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>922</v>
+        <v>587</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>923</v>
+        <v>588</v>
       </c>
     </row>
     <row r="21">
@@ -20124,10 +20315,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>924</v>
+        <v>589</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>925</v>
+        <v>590</v>
       </c>
     </row>
     <row r="22">
@@ -20135,10 +20326,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>926</v>
+        <v>914</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>927</v>
+        <v>915</v>
       </c>
     </row>
     <row r="23">
@@ -20146,10 +20337,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>928</v>
+        <v>916</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>929</v>
+        <v>917</v>
       </c>
     </row>
     <row r="24">
@@ -20157,10 +20348,10 @@
         <v>21</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>928</v>
+        <v>918</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>929</v>
+        <v>919</v>
       </c>
     </row>
     <row r="25">
@@ -20168,10 +20359,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>930</v>
+        <v>724</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>931</v>
+        <v>725</v>
       </c>
     </row>
     <row r="26">
@@ -20179,10 +20370,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>932</v>
+        <v>920</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>933</v>
+        <v>921</v>
       </c>
     </row>
     <row r="27">
@@ -20190,10 +20381,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>932</v>
+        <v>922</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>933</v>
+        <v>923</v>
       </c>
     </row>
     <row r="28">
@@ -20201,10 +20392,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>722</v>
+        <v>924</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>723</v>
+        <v>925</v>
       </c>
     </row>
     <row r="29">
@@ -20212,10 +20403,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>595</v>
+        <v>14</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>596</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30">
@@ -20223,10 +20414,10 @@
         <v>27</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>934</v>
+        <v>14</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>935</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31">
@@ -20234,10 +20425,10 @@
         <v>28</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>934</v>
+        <v>14</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>935</v>
+        <v>15</v>
       </c>
     </row>
     <row r="32">
@@ -20245,10 +20436,10 @@
         <v>29</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>936</v>
+        <v>14</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>937</v>
+        <v>15</v>
       </c>
     </row>
     <row r="33">
@@ -20256,10 +20447,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>299</v>
+        <v>14</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>300</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34">
@@ -20267,10 +20458,10 @@
         <v>31</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>408</v>
+        <v>926</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>409</v>
+        <v>927</v>
       </c>
     </row>
     <row r="35">
@@ -20278,10 +20469,10 @@
         <v>32</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>14</v>
+        <v>410</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>15</v>
+        <v>411</v>
       </c>
     </row>
     <row r="36">
@@ -20289,10 +20480,10 @@
         <v>33</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>14</v>
+        <v>53</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>15</v>
+        <v>54</v>
       </c>
     </row>
     <row r="37">
@@ -20300,10 +20491,10 @@
         <v>34</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="38">
@@ -20311,10 +20502,10 @@
         <v>35</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>14</v>
+        <v>928</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>15</v>
+        <v>929</v>
       </c>
     </row>
     <row r="39">
@@ -20322,10 +20513,10 @@
         <v>36</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>14</v>
+        <v>666</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>15</v>
+        <v>667</v>
       </c>
     </row>
     <row r="40">
@@ -20333,10 +20524,10 @@
         <v>37</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>14</v>
+        <v>930</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>15</v>
+        <v>931</v>
       </c>
     </row>
     <row r="41">
@@ -20344,10 +20535,10 @@
         <v>38</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>938</v>
+        <v>97</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>939</v>
+        <v>98</v>
       </c>
     </row>
     <row r="42">
@@ -20355,10 +20546,10 @@
         <v>39</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>938</v>
+        <v>97</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>939</v>
+        <v>98</v>
       </c>
     </row>
     <row r="43">
@@ -20366,10 +20557,10 @@
         <v>40</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>410</v>
+        <v>932</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>411</v>
+        <v>933</v>
       </c>
     </row>
     <row r="44">
@@ -20377,10 +20568,10 @@
         <v>41</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>410</v>
+        <v>103</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>411</v>
+        <v>104</v>
       </c>
     </row>
     <row r="45">
@@ -20388,10 +20579,10 @@
         <v>42</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>940</v>
+        <v>103</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>941</v>
+        <v>104</v>
       </c>
     </row>
     <row r="46">
@@ -20399,10 +20590,10 @@
         <v>43</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>942</v>
+        <v>22</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>943</v>
+        <v>23</v>
       </c>
     </row>
     <row r="47">
@@ -20410,10 +20601,10 @@
         <v>44</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>944</v>
+        <v>22</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>945</v>
+        <v>23</v>
       </c>
     </row>
     <row r="48">
@@ -20421,10 +20612,10 @@
         <v>45</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>944</v>
+        <v>225</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>945</v>
+        <v>226</v>
       </c>
     </row>
     <row r="49">
@@ -20432,10 +20623,10 @@
         <v>46</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>148</v>
+        <v>30</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>149</v>
+        <v>31</v>
       </c>
     </row>
     <row r="50">
@@ -20443,10 +20634,10 @@
         <v>47</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>53</v>
+        <v>934</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>54</v>
+        <v>935</v>
       </c>
     </row>
     <row r="51">
@@ -20454,10 +20645,10 @@
         <v>48</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>18</v>
+        <v>936</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>19</v>
+        <v>937</v>
       </c>
     </row>
     <row r="52">
@@ -20465,10 +20656,10 @@
         <v>49</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>55</v>
+        <v>938</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>56</v>
+        <v>939</v>
       </c>
     </row>
     <row r="53">
@@ -20476,10 +20667,10 @@
         <v>50</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>55</v>
+        <v>940</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>56</v>
+        <v>235</v>
       </c>
     </row>
     <row r="54">
@@ -20487,10 +20678,10 @@
         <v>51</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>55</v>
+        <v>162</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>56</v>
+        <v>163</v>
       </c>
     </row>
     <row r="55">
@@ -20498,10 +20689,10 @@
         <v>52</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
     </row>
     <row r="56">
@@ -20509,10 +20700,10 @@
         <v>53</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
     </row>
     <row r="57">
@@ -20520,10 +20711,10 @@
         <v>54</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>946</v>
+        <v>129</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>947</v>
+        <v>130</v>
       </c>
     </row>
     <row r="58">
@@ -20531,10 +20722,10 @@
         <v>55</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>946</v>
+        <v>44</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>947</v>
+        <v>45</v>
       </c>
     </row>
     <row r="59">
@@ -20542,10 +20733,10 @@
         <v>56</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>103</v>
+        <v>46</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>104</v>
+        <v>47</v>
       </c>
     </row>
     <row r="60">
@@ -20553,10 +20744,10 @@
         <v>57</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>103</v>
+        <v>696</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>104</v>
+        <v>697</v>
       </c>
     </row>
     <row r="61">
@@ -20564,10 +20755,10 @@
         <v>58</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>948</v>
+        <v>696</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>949</v>
+        <v>697</v>
       </c>
     </row>
     <row r="62">
@@ -20575,10 +20766,10 @@
         <v>59</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>948</v>
+        <v>619</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>949</v>
+        <v>620</v>
       </c>
     </row>
     <row r="63">
@@ -20586,10 +20777,10 @@
         <v>60</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>948</v>
+        <v>943</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>949</v>
+        <v>944</v>
       </c>
     </row>
     <row r="64">
@@ -20597,362 +20788,10 @@
         <v>61</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>948</v>
+        <v>945</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>949</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="3">
-        <v>62</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>634</v>
-      </c>
-      <c r="C65" s="4" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="3">
-        <v>63</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>634</v>
-      </c>
-      <c r="C66" s="4" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="3">
-        <v>64</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>465</v>
-      </c>
-      <c r="C67" s="4" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="3">
-        <v>65</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>465</v>
-      </c>
-      <c r="C68" s="4" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="3">
-        <v>66</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="C69" s="4" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="3">
-        <v>67</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C70" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="3">
-        <v>68</v>
-      </c>
-      <c r="B71" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C71" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="3">
-        <v>69</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>566</v>
-      </c>
-      <c r="C72" s="4" t="s">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="3">
-        <v>70</v>
-      </c>
-      <c r="B73" s="3" t="s">
-        <v>950</v>
-      </c>
-      <c r="C73" s="4" t="s">
-        <v>951</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="3">
-        <v>71</v>
-      </c>
-      <c r="B74" s="3" t="s">
-        <v>952</v>
-      </c>
-      <c r="C74" s="4" t="s">
-        <v>953</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="3">
-        <v>72</v>
-      </c>
-      <c r="B75" s="3" t="s">
-        <v>954</v>
-      </c>
-      <c r="C75" s="4" t="s">
-        <v>955</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="3">
-        <v>73</v>
-      </c>
-      <c r="B76" s="3" t="s">
-        <v>956</v>
-      </c>
-      <c r="C76" s="4" t="s">
-        <v>957</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="3">
-        <v>74</v>
-      </c>
-      <c r="B77" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C77" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="3">
-        <v>75</v>
-      </c>
-      <c r="B78" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C78" s="4" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="3">
-        <v>76</v>
-      </c>
-      <c r="B79" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C79" s="4" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="3">
-        <v>77</v>
-      </c>
-      <c r="B80" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C80" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="3">
-        <v>78</v>
-      </c>
-      <c r="B81" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C81" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="3">
-        <v>79</v>
-      </c>
-      <c r="B82" s="3" t="s">
-        <v>958</v>
-      </c>
-      <c r="C82" s="4" t="s">
-        <v>959</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="3">
-        <v>80</v>
-      </c>
-      <c r="B83" s="3" t="s">
-        <v>958</v>
-      </c>
-      <c r="C83" s="4" t="s">
-        <v>959</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="3">
-        <v>81</v>
-      </c>
-      <c r="B84" s="3" t="s">
-        <v>960</v>
-      </c>
-      <c r="C84" s="4" t="s">
-        <v>961</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="3">
-        <v>82</v>
-      </c>
-      <c r="B85" s="3" t="s">
-        <v>962</v>
-      </c>
-      <c r="C85" s="4" t="s">
-        <v>963</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="3">
-        <v>83</v>
-      </c>
-      <c r="B86" s="3" t="s">
-        <v>964</v>
-      </c>
-      <c r="C86" s="4" t="s">
-        <v>965</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="3">
-        <v>84</v>
-      </c>
-      <c r="B87" s="3" t="s">
-        <v>966</v>
-      </c>
-      <c r="C87" s="4" t="s">
-        <v>967</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="3">
-        <v>85</v>
-      </c>
-      <c r="B88" s="3" t="s">
-        <v>968</v>
-      </c>
-      <c r="C88" s="4" t="s">
-        <v>969</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="3">
-        <v>86</v>
-      </c>
-      <c r="B89" s="3" t="s">
-        <v>970</v>
-      </c>
-      <c r="C89" s="4" t="s">
-        <v>971</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="3">
-        <v>87</v>
-      </c>
-      <c r="B90" s="3" t="s">
-        <v>972</v>
-      </c>
-      <c r="C90" s="4" t="s">
-        <v>973</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="3">
-        <v>88</v>
-      </c>
-      <c r="B91" s="3" t="s">
-        <v>972</v>
-      </c>
-      <c r="C91" s="4" t="s">
-        <v>973</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="3">
-        <v>89</v>
-      </c>
-      <c r="B92" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="C92" s="4" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="3">
-        <v>90</v>
-      </c>
-      <c r="B93" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C93" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="3">
-        <v>91</v>
-      </c>
-      <c r="B94" s="3" t="s">
-        <v>974</v>
-      </c>
-      <c r="C94" s="4" t="s">
-        <v>975</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="3">
-        <v>92</v>
-      </c>
-      <c r="B95" s="3" t="s">
-        <v>976</v>
-      </c>
-      <c r="C95" s="4" t="s">
-        <v>977</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="3">
-        <v>93</v>
-      </c>
-      <c r="B96" s="3" t="s">
-        <v>978</v>
-      </c>
-      <c r="C96" s="4" t="s">
-        <v>979</v>
+        <v>946</v>
       </c>
     </row>
   </sheetData>
@@ -20961,7 +20800,7 @@
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>
@@ -20972,16 +20811,16 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
-    <col customWidth="1" min="3" max="3" width="60"/>
+    <col customWidth="1" min="3" max="3" width="69.140625"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="21">
       <c r="A1" s="1" t="s">
-        <v>980</v>
+        <v>947</v>
       </c>
     </row>
     <row r="3">
@@ -21000,10 +20839,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>4</v>
+        <v>699</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>5</v>
+        <v>700</v>
       </c>
     </row>
     <row r="5">
@@ -21011,10 +20850,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>6</v>
+        <v>136</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>7</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6">
@@ -21022,10 +20861,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>6</v>
+        <v>405</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>7</v>
+        <v>406</v>
       </c>
     </row>
     <row r="7">
@@ -21033,10 +20872,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8">
@@ -21044,10 +20883,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9">
@@ -21055,10 +20894,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>981</v>
+        <v>6</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>235</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -21066,10 +20905,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>272</v>
+        <v>79</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>235</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11">
@@ -21077,10 +20916,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12">
@@ -21088,10 +20927,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>85</v>
+        <v>948</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>86</v>
+        <v>949</v>
       </c>
     </row>
     <row r="13">
@@ -21099,10 +20938,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>982</v>
+        <v>950</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>983</v>
+        <v>951</v>
       </c>
     </row>
     <row r="14">
@@ -21110,10 +20949,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>14</v>
+        <v>952</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>15</v>
+        <v>953</v>
       </c>
     </row>
     <row r="15">
@@ -21121,10 +20960,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>14</v>
+        <v>954</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>15</v>
+        <v>955</v>
       </c>
     </row>
     <row r="16">
@@ -21132,10 +20971,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>14</v>
+        <v>571</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>15</v>
+        <v>572</v>
       </c>
     </row>
     <row r="17">
@@ -21143,10 +20982,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>14</v>
+        <v>956</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>15</v>
+        <v>957</v>
       </c>
     </row>
     <row r="18">
@@ -21154,10 +20993,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>14</v>
+        <v>272</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>15</v>
+        <v>235</v>
       </c>
     </row>
     <row r="19">
@@ -21165,10 +21004,10 @@
         <v>16</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>14</v>
+        <v>273</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>15</v>
+        <v>274</v>
       </c>
     </row>
     <row r="20">
@@ -21176,10 +21015,10 @@
         <v>17</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>146</v>
+        <v>912</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>147</v>
+        <v>913</v>
       </c>
     </row>
     <row r="21">
@@ -21187,10 +21026,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>410</v>
+        <v>585</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>411</v>
+        <v>586</v>
       </c>
     </row>
     <row r="22">
@@ -21198,10 +21037,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>51</v>
+        <v>585</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>52</v>
+        <v>586</v>
       </c>
     </row>
     <row r="23">
@@ -21209,10 +21048,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>18</v>
+        <v>587</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>19</v>
+        <v>588</v>
       </c>
     </row>
     <row r="24">
@@ -21220,10 +21059,10 @@
         <v>21</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>412</v>
+        <v>589</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>413</v>
+        <v>590</v>
       </c>
     </row>
     <row r="25">
@@ -21231,10 +21070,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>412</v>
+        <v>916</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>413</v>
+        <v>917</v>
       </c>
     </row>
     <row r="26">
@@ -21242,10 +21081,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>55</v>
+        <v>724</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>56</v>
+        <v>725</v>
       </c>
     </row>
     <row r="27">
@@ -21253,10 +21092,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>55</v>
+        <v>724</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>56</v>
+        <v>725</v>
       </c>
     </row>
     <row r="28">
@@ -21264,10 +21103,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>22</v>
+        <v>922</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>23</v>
+        <v>923</v>
       </c>
     </row>
     <row r="29">
@@ -21275,10 +21114,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>22</v>
+        <v>924</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>23</v>
+        <v>925</v>
       </c>
     </row>
     <row r="30">
@@ -21286,10 +21125,10 @@
         <v>27</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31">
@@ -21297,10 +21136,10 @@
         <v>28</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="32">
@@ -21308,10 +21147,10 @@
         <v>29</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
     </row>
     <row r="33">
@@ -21319,10 +21158,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34">
@@ -21330,10 +21169,10 @@
         <v>31</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>107</v>
+        <v>14</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>108</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35">
@@ -21341,10 +21180,10 @@
         <v>32</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>67</v>
+        <v>926</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>68</v>
+        <v>927</v>
       </c>
     </row>
     <row r="36">
@@ -21352,10 +21191,10 @@
         <v>33</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>67</v>
+        <v>958</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>68</v>
+        <v>959</v>
       </c>
     </row>
     <row r="37">
@@ -21363,10 +21202,10 @@
         <v>34</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>179</v>
+        <v>296</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>180</v>
+        <v>297</v>
       </c>
     </row>
     <row r="38">
@@ -21374,10 +21213,10 @@
         <v>35</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>111</v>
+        <v>16</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>112</v>
+        <v>17</v>
       </c>
     </row>
     <row r="39">
@@ -21385,10 +21224,10 @@
         <v>36</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>112</v>
+        <v>94</v>
       </c>
     </row>
     <row r="40">
@@ -21396,10 +21235,10 @@
         <v>37</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>111</v>
+        <v>960</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>112</v>
+        <v>961</v>
       </c>
     </row>
     <row r="41">
@@ -21407,10 +21246,10 @@
         <v>38</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>59</v>
+        <v>97</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>60</v>
+        <v>98</v>
       </c>
     </row>
     <row r="42">
@@ -21418,10 +21257,10 @@
         <v>39</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>38</v>
+        <v>932</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>39</v>
+        <v>933</v>
       </c>
     </row>
     <row r="43">
@@ -21429,10 +21268,10 @@
         <v>40</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>414</v>
+        <v>103</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>415</v>
+        <v>104</v>
       </c>
     </row>
     <row r="44">
@@ -21440,10 +21279,10 @@
         <v>41</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>984</v>
+        <v>22</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>985</v>
+        <v>23</v>
       </c>
     </row>
     <row r="45">
@@ -21451,10 +21290,10 @@
         <v>42</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>986</v>
+        <v>22</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>987</v>
+        <v>23</v>
       </c>
     </row>
     <row r="46">
@@ -21462,10 +21301,10 @@
         <v>43</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>988</v>
+        <v>225</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>989</v>
+        <v>226</v>
       </c>
     </row>
     <row r="47">
@@ -21473,10 +21312,10 @@
         <v>44</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>988</v>
+        <v>30</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>989</v>
+        <v>31</v>
       </c>
     </row>
     <row r="48">
@@ -21484,10 +21323,10 @@
         <v>45</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>123</v>
+        <v>934</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>124</v>
+        <v>935</v>
       </c>
     </row>
     <row r="49">
@@ -21495,10 +21334,10 @@
         <v>46</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>40</v>
+        <v>936</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>41</v>
+        <v>937</v>
       </c>
     </row>
     <row r="50">
@@ -21506,10 +21345,10 @@
         <v>47</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>125</v>
+        <v>938</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>126</v>
+        <v>939</v>
       </c>
     </row>
     <row r="51">
@@ -21517,10 +21356,10 @@
         <v>48</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>166</v>
+        <v>615</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>167</v>
+        <v>616</v>
       </c>
     </row>
     <row r="52">
@@ -21528,10 +21367,10 @@
         <v>49</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>128</v>
+        <v>163</v>
       </c>
     </row>
     <row r="53">
@@ -21539,10 +21378,10 @@
         <v>50</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>127</v>
+        <v>40</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>128</v>
+        <v>41</v>
       </c>
     </row>
     <row r="54">
@@ -21550,10 +21389,10 @@
         <v>51</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>129</v>
+        <v>941</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>130</v>
+        <v>942</v>
       </c>
     </row>
     <row r="55">
@@ -21561,10 +21400,10 @@
         <v>52</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>990</v>
+        <v>44</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>235</v>
+        <v>45</v>
       </c>
     </row>
     <row r="56">
@@ -21572,10 +21411,10 @@
         <v>53</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>991</v>
+        <v>46</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>992</v>
+        <v>47</v>
       </c>
     </row>
     <row r="57">
@@ -21583,10 +21422,10 @@
         <v>54</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>991</v>
+        <v>696</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>992</v>
+        <v>697</v>
       </c>
     </row>
     <row r="58">
@@ -21594,10 +21433,32 @@
         <v>55</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>46</v>
+        <v>696</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>47</v>
+        <v>697</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3">
+        <v>56</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>943</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3">
+        <v>57</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>945</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>946</v>
       </c>
     </row>
   </sheetData>
@@ -21617,6 +21478,1714 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="8"/>
+    <col customWidth="1" min="2" max="2" width="15"/>
+    <col customWidth="1" min="3" max="3" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>962</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>963</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>965</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>966</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>8</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>967</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>969</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3">
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>971</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>973</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>974</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>975</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>977</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3">
+        <v>14</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>979</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>980</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3">
+        <v>15</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>981</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3">
+        <v>16</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>983</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>985</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>986</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>987</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3">
+        <v>19</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>989</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3">
+        <v>20</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>991</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>991</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3">
+        <v>22</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>993</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3">
+        <v>23</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>995</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3">
+        <v>24</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>995</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3">
+        <v>25</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>722</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3">
+        <v>26</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3">
+        <v>27</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>918</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3">
+        <v>28</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>918</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3">
+        <v>29</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3">
+        <v>30</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3">
+        <v>31</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3">
+        <v>32</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3">
+        <v>33</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3">
+        <v>34</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3">
+        <v>35</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3">
+        <v>36</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3">
+        <v>37</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3">
+        <v>38</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>999</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3">
+        <v>39</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>999</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3">
+        <v>40</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3">
+        <v>41</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3">
+        <v>42</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3">
+        <v>43</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3">
+        <v>44</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>1005</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3">
+        <v>45</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>1005</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3">
+        <v>46</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3">
+        <v>47</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3">
+        <v>48</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3">
+        <v>49</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3">
+        <v>50</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3">
+        <v>51</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3">
+        <v>52</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3">
+        <v>53</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>1007</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3">
+        <v>54</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>1007</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3">
+        <v>55</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>1007</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3">
+        <v>56</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3">
+        <v>57</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3">
+        <v>58</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>1009</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3">
+        <v>59</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>1009</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3">
+        <v>60</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>1009</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3">
+        <v>61</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>1009</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3">
+        <v>62</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3">
+        <v>63</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3">
+        <v>64</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3">
+        <v>65</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3">
+        <v>66</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3">
+        <v>67</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3">
+        <v>68</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3">
+        <v>69</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>566</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3">
+        <v>70</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3">
+        <v>71</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3">
+        <v>72</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>1015</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3">
+        <v>73</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>1017</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3">
+        <v>74</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3">
+        <v>75</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3">
+        <v>76</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3">
+        <v>77</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3">
+        <v>78</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3">
+        <v>79</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3">
+        <v>80</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3">
+        <v>81</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3">
+        <v>82</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3">
+        <v>83</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>1025</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3">
+        <v>84</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3">
+        <v>85</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>1029</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3">
+        <v>86</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>1031</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3">
+        <v>87</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3">
+        <v>88</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3">
+        <v>89</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3">
+        <v>90</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3">
+        <v>91</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>1035</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3">
+        <v>92</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>1037</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3">
+        <v>93</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>1039</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>1040</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="8"/>
+    <col customWidth="1" min="2" max="2" width="15"/>
+    <col customWidth="1" min="3" max="3" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>8</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3">
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>1043</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3">
+        <v>14</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3">
+        <v>15</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3">
+        <v>16</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3">
+        <v>19</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3">
+        <v>20</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3">
+        <v>22</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3">
+        <v>23</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3">
+        <v>24</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3">
+        <v>25</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3">
+        <v>26</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3">
+        <v>27</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3">
+        <v>28</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3">
+        <v>29</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3">
+        <v>30</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3">
+        <v>31</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3">
+        <v>32</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3">
+        <v>33</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3">
+        <v>34</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3">
+        <v>35</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3">
+        <v>36</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3">
+        <v>37</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3">
+        <v>38</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3">
+        <v>39</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3">
+        <v>40</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3">
+        <v>41</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>1045</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>1046</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3">
+        <v>42</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>1047</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3">
+        <v>43</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3">
+        <v>44</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3">
+        <v>45</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3">
+        <v>46</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3">
+        <v>47</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3">
+        <v>48</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3">
+        <v>49</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3">
+        <v>50</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3">
+        <v>51</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3">
+        <v>52</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>1049</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3">
+        <v>53</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>1050</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3">
+        <v>54</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>1050</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3">
+        <v>55</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
@@ -21626,7 +23195,7 @@
   <sheetData>
     <row r="1" ht="21">
       <c r="A1" s="1" t="s">
-        <v>993</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="3">
@@ -21810,10 +23379,10 @@
         <v>16</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>994</v>
+        <v>1053</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>995</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="20">
@@ -21865,10 +23434,10 @@
         <v>21</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>996</v>
+        <v>1055</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>997</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="25">
@@ -21876,10 +23445,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>996</v>
+        <v>1055</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>997</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="26">
@@ -21898,10 +23467,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>998</v>
+        <v>1057</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>999</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="28">
@@ -21975,10 +23544,10 @@
         <v>31</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>1000</v>
+        <v>1059</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>1001</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="35">
@@ -22019,10 +23588,10 @@
         <v>35</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>956</v>
+        <v>1017</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>957</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="39">
@@ -22096,10 +23665,10 @@
         <v>42</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>1002</v>
+        <v>1061</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>1003</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="46">
@@ -22107,10 +23676,10 @@
         <v>43</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>1002</v>
+        <v>1061</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>1003</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="47">
@@ -22118,10 +23687,10 @@
         <v>44</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>1002</v>
+        <v>1061</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>1003</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="48">
@@ -22129,10 +23698,10 @@
         <v>45</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>1004</v>
+        <v>1063</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>1005</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="49">
@@ -22155,6 +23724,266 @@
       </c>
       <c r="C50" s="4" t="s">
         <v>476</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="8"/>
+    <col customWidth="1" min="2" max="2" width="15"/>
+    <col customWidth="1" min="3" max="3" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>8</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3">
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3">
+        <v>14</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3">
+        <v>15</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3">
+        <v>16</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3">
+        <v>19</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3">
+        <v>20</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>493</v>
       </c>
     </row>
   </sheetData>
@@ -22560,6 +24389,471 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="8"/>
+    <col customWidth="1" min="2" max="2" width="15"/>
+    <col customWidth="1" min="3" max="3" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>8</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3">
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3">
+        <v>14</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3">
+        <v>15</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3">
+        <v>16</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3">
+        <v>19</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>493</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="8"/>
+    <col customWidth="1" min="2" max="2" width="15"/>
+    <col customWidth="1" min="3" max="3" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>8</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3">
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3">
+        <v>14</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3">
+        <v>15</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3">
+        <v>16</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>493</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>

</xml_diff>

<commit_message>
Adénome Prostate AP 1
</commit_message>
<xml_diff>
--- a/public/instruments_inventory.xlsx
+++ b/public/instruments_inventory.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="52" showHorizontalScroll="1" showVerticalScroll="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="53" showHorizontalScroll="1" showVerticalScroll="1"/>
   </bookViews>
   <sheets>
     <sheet name="CESARIENNE 2" sheetId="1" state="visible" r:id="rId1"/>
@@ -60,6 +60,7 @@
     <sheet name="CURETTAGE 4" sheetId="51" state="visible" r:id="rId51"/>
     <sheet name="FAV 1" sheetId="52" state="visible" r:id="rId52"/>
     <sheet name="ENDOSCOPIE HYPOPHYSE 1" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="ADENOME PROSTATE (AP) 1" sheetId="54" state="visible" r:id="rId54"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
   <extLst>
@@ -69,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1113" uniqueCount="1113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1123" uniqueCount="1123">
   <si>
     <t xml:space="preserve">CESARIENNE 2</t>
   </si>
@@ -3408,6 +3409,36 @@
   </si>
   <si>
     <t xml:space="preserve">PINCE ORL RHINO WEIL BLAKESLEY 125 X 3,5 MM CDE HT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADENOME PROSTATE (AP) 1</t>
+  </si>
+  <si>
+    <t>20902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECARTEUR ABDOM. GOSSET AV CREM. 45 X 60 X 200</t>
+  </si>
+  <si>
+    <t>21103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECARTEUR ABDOM. JUDD MASSON COMPLET</t>
+  </si>
+  <si>
+    <t>34103</t>
+  </si>
+  <si>
+    <t>38916</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PINCE PREHENS. MULTIGR. THOMS ALLIS  200 MM  6 X 7</t>
+  </si>
+  <si>
+    <t>47502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALVE LERICHE BUGATTI            35 X 210 MM</t>
   </si>
 </sst>
 </file>
@@ -24997,14 +25028,14 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
     <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>1068</v>
       </c>
@@ -25455,7 +25486,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="8"/>
     <col customWidth="1" min="2" max="2" width="15"/>
-    <col customWidth="1" min="3" max="3" width="69.00390625"/>
+    <col customWidth="1" min="3" max="3" width="60"/>
   </cols>
   <sheetData>
     <row r="1" ht="21">
@@ -25855,6 +25886,574 @@
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="8"/>
+    <col customWidth="1" min="2" max="2" width="15"/>
+    <col customWidth="1" min="3" max="3" width="69.28125"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="21">
+      <c r="A1" s="1" t="s">
+        <v>1113</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>1114</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>1115</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>8</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>1117</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3">
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3">
+        <v>14</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3">
+        <v>15</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3">
+        <v>16</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3">
+        <v>19</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3">
+        <v>20</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>1118</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3">
+        <v>22</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3">
+        <v>23</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3">
+        <v>24</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3">
+        <v>25</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3">
+        <v>26</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3">
+        <v>27</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3">
+        <v>28</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3">
+        <v>29</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3">
+        <v>30</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3">
+        <v>31</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3">
+        <v>32</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3">
+        <v>33</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3">
+        <v>34</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3">
+        <v>35</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3">
+        <v>36</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3">
+        <v>37</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3">
+        <v>38</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3">
+        <v>39</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>1121</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>1122</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3">
+        <v>40</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3">
+        <v>41</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3">
+        <v>42</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3">
+        <v>43</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3">
+        <v>44</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3">
+        <v>45</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3">
+        <v>46</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3">
+        <v>47</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3">
+        <v>48</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.29999999999999999" right="0" top="0.29999999999999999" bottom="0" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" scale="109" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>

</xml_diff>